<commit_message>
modify Excel in EuRoC_rapport
</commit_message>
<xml_diff>
--- a/RocketPy_26/EuRoC_rapport/EuRoC_rapport.xlsx
+++ b/RocketPy_26/EuRoC_rapport/EuRoC_rapport.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="768" yWindow="0" windowWidth="11712" windowHeight="12240" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" state="visible" r:id="rId1"/>
@@ -233,7 +233,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -281,6 +281,7 @@
     </xf>
     <xf numFmtId="165" fontId="8" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="9" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -1697,8 +1698,8 @@
   <mergeCells count="15">
     <mergeCell ref="A41:C41"/>
     <mergeCell ref="A47:C47"/>
+    <mergeCell ref="A14:C14"/>
     <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A14:C14"/>
     <mergeCell ref="A58:C58"/>
     <mergeCell ref="A17:C17"/>
     <mergeCell ref="A67:C67"/>
@@ -1722,7 +1723,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C40"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4"/>
   <cols>
     <col width="32" customWidth="1" style="20" min="1" max="1"/>
@@ -1947,212 +1948,257 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>m_eth_density</t>
+          <t>eth_temperature</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>810</v>
+        <v>293.15</v>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Masse volumique eth </t>
+          <t>Température en K</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>m_lox_unused</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>0.577</v>
+          <t>eth_pressure</t>
+        </is>
+      </c>
+      <c r="B22" s="27" t="n">
+        <v>6000000</v>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lox non-consommé </t>
+          <t>Pression en Pa</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>m_lox_density</t>
+          <t>eth_massic_frac</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>1154</v>
+        <v>0.9</v>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Masse volumique lox</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="20">
+          <t>Fraction massique de l'eth dans le fuel (par rapport à l'eau)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>m_n2</t>
+          <t>m_lox_unused</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>2.605</v>
+        <v>0.577</v>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">N2 dans un copv </t>
+          <t xml:space="preserve">Lox non-consommé </t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="21" t="inlineStr">
-        <is>
-          <t>TIME</t>
-        </is>
-      </c>
-      <c r="B25" s="22" t="n"/>
-      <c r="C25" s="22" t="n"/>
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>lox_temperature</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>90.15000000000001</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Température en K</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">hold_time </t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="27">
+          <t>lox_pressure</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Pression en Pa</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="15" customHeight="1" s="20">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">prechill_time </t>
+          <t>m_n2</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>0.2</v>
+        <v>2.605</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N2 dans un copv </t>
+        </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>ignition_delay</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>0.13</v>
-      </c>
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>TIME</t>
+        </is>
+      </c>
+      <c r="B28" s="22" t="n"/>
+      <c r="C28" s="22" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">ramp_up_time </t>
+          <t xml:space="preserve">hold_time </t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>0.125</v>
+        <v>300</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">cutoff_time </t>
+          <t xml:space="preserve">prechill_time </t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>0.04</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">ramp_down_time </t>
+          <t>ignition_delay</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>0.175</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FORCE </t>
-        </is>
-      </c>
-      <c r="B32" s="22" t="n"/>
-      <c r="C32" s="22" t="n"/>
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ramp_up_time </t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>0.125</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">f_shutdown </t>
+          <t xml:space="preserve">cutoff_time </t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>0</v>
-      </c>
-      <c r="C33" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Force finale de la thrust curve </t>
-        </is>
+        <v>0.04</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">f_hold_down </t>
+          <t xml:space="preserve">ramp_down_time </t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>4500</v>
-      </c>
-      <c r="C34" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Force du hold-down </t>
-        </is>
+        <v>0.175</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="23" t="inlineStr">
-        <is>
-          <t>THRUST CURVE MODEL</t>
-        </is>
-      </c>
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FORCE </t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="22" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>thrust_curve_mode</t>
-        </is>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>constant</t>
-        </is>
+          <t xml:space="preserve">f_shutdown </t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>0</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>constant or peaked</t>
+          <t xml:space="preserve">Force finale de la thrust curve </t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t xml:space="preserve">f_hold_down </t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>4500</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Force du hold-down </t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="23" t="inlineStr">
+        <is>
+          <t>THRUST CURVE MODEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>thrust_curve_mode</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>constant</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>constant or peaked</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
           <t>derated_thrust</t>
         </is>
       </c>
-      <c r="B37" t="n">
+      <c r="B40" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A38:C38"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2581,7 +2627,7 @@
       <c r="B1" s="7" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="27" t="inlineStr">
+      <c r="A2" s="28" t="inlineStr">
         <is>
           <t>MASSE</t>
         </is>
@@ -2608,7 +2654,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>PERFORMANCES MOTEUR</t>
         </is>
@@ -2621,7 +2667,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>7000</v>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -2635,7 +2681,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>CINÉMATIQUE &amp; TRAJECTOIRE</t>
         </is>
@@ -2648,7 +2694,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>3117.467115177918</v>
+        <v>3109.373713103756</v>
       </c>
     </row>
     <row r="10">
@@ -2658,7 +2704,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>3276.467115177918</v>
+        <v>3277.373713103756</v>
       </c>
     </row>
     <row r="11">
@@ -2668,7 +2714,7 @@
         </is>
       </c>
       <c r="B11" s="5" t="n">
-        <v>251.3657654310787</v>
+        <v>249.3429892488362</v>
       </c>
     </row>
     <row r="12">
@@ -2678,7 +2724,7 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>147.9734383829405</v>
+        <v>125.6674940708535</v>
       </c>
     </row>
     <row r="13">
@@ -2688,7 +2734,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>0.7287446459365355</v>
+        <v>0.7381918825994666</v>
       </c>
     </row>
     <row r="14">
@@ -2698,7 +2744,7 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>26.94485805142876</v>
+        <v>26.93569684002304</v>
       </c>
     </row>
     <row r="15">
@@ -2708,11 +2754,11 @@
         </is>
       </c>
       <c r="B15" s="5" t="n">
-        <v>231.8870545311422</v>
+        <v>234.1582721970778</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>SORTIE DE RAMPE</t>
         </is>
@@ -2725,7 +2771,7 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>32.43710250281957</v>
+        <v>32.4325676450251</v>
       </c>
     </row>
     <row r="18">
@@ -2735,11 +2781,11 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>4.047917040148098</v>
+        <v>4.047491964508415</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>STABILITÉ</t>
         </is>
@@ -2752,7 +2798,7 @@
         </is>
       </c>
       <c r="B20" s="10" t="n">
-        <v>4.014143199086379</v>
+        <v>4.013504246372449</v>
       </c>
     </row>
     <row r="21" ht="14.7" customHeight="1" s="20">

</xml_diff>

<commit_message>
create new column for the masses in the case CoM == 1
</commit_message>
<xml_diff>
--- a/RocketPy_26/EuRoC_rapport/EuRoC_rapport.xlsx
+++ b/RocketPy_26/EuRoC_rapport/EuRoC_rapport.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1260" yWindow="2328" windowWidth="17280" windowHeight="9960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" state="visible" r:id="rId1"/>
@@ -12,7 +12,7 @@
     <sheet name="Simulation" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="171027" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -24,7 +24,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -63,12 +63,6 @@
     </font>
     <font>
       <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
       <sz val="10"/>
     </font>
     <font>
@@ -78,8 +72,20 @@
       <color theme="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFFFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -126,12 +132,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F497D"/>
-        <bgColor rgb="001F497D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFCCCCCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -140,6 +140,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFEFEFEF"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1F497D"/>
+        <bgColor rgb="FF1F497D"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+        <bgColor rgb="001F497D"/>
       </patternFill>
     </fill>
   </fills>
@@ -216,7 +228,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -233,39 +245,44 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="11" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="8" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -631,16 +648,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.77734375" defaultRowHeight="14.4" customHeight="1" outlineLevelRow="0"/>
+  <dimension ref="A1:I75"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
-    <col width="32" customWidth="1" style="1" min="1" max="1"/>
-    <col width="16" customWidth="1" style="1" min="2" max="2"/>
-    <col width="55" customWidth="1" style="1" min="3" max="3"/>
-    <col width="10.44140625" customWidth="1" style="1" min="5" max="5"/>
+    <col width="32" customWidth="1" style="23" min="1" max="1"/>
+    <col width="16" customWidth="1" style="23" min="2" max="2"/>
+    <col width="55" customWidth="1" style="23" min="3" max="3"/>
+    <col width="32.33203125" bestFit="1" customWidth="1" min="4" max="4"/>
+    <col width="10.44140625" customWidth="1" style="23" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.05" customFormat="1" customHeight="1" s="1">
+    <row r="1" ht="22.05" customFormat="1" customHeight="1" s="23">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Name</t>
@@ -656,23 +674,30 @@
           <t>Description</t>
         </is>
       </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Value (mass) for mode_CoM == 1</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">ROCKET </t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="D2" s="22" t="n"/>
+      <c r="E2" s="23" t="n"/>
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Longeur :</t>
         </is>
       </c>
-      <c r="F2">
+      <c r="G2">
         <f>B12+B16+B20+B29+B33+B37+B40+B43+B49</f>
         <v/>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>[m]</t>
         </is>
@@ -685,14 +710,14 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
           <t>0 or 1</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -708,16 +733,16 @@
           <t>0 or 1</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Dry mass: </t>
         </is>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <f>SUM(B13,B17,B21,B24,B30,B34,B38,B41,B44,B50)+B67</f>
         <v/>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>[kg]</t>
         </is>
@@ -737,9 +762,9 @@
           <t>Mode 1 only</t>
         </is>
       </c>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5">
-        <f>F4+B6</f>
+      <c r="F5" s="4" t="n"/>
+      <c r="G5">
+        <f>G4+B6</f>
         <v/>
       </c>
     </row>
@@ -757,7 +782,7 @@
           <t>Mode 1 only</t>
         </is>
       </c>
-      <c r="E6" s="7" t="n"/>
+      <c r="F6" s="7" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -773,11 +798,11 @@
           <t xml:space="preserve">Rayon  </t>
         </is>
       </c>
-      <c r="E7">
+      <c r="F7">
         <f>B7*2</f>
         <v/>
       </c>
-      <c r="H7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -795,11 +820,12 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">BOAT TAIL </t>
         </is>
       </c>
+      <c r="D9" s="22" t="n"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -863,7 +889,7 @@
       <c r="D13" t="n">
         <v>1.05</v>
       </c>
-      <c r="E13" t="n">
+      <c r="F13" t="n">
         <v>7.353</v>
       </c>
     </row>
@@ -883,11 +909,12 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>ENGINE BAY</t>
         </is>
       </c>
+      <c r="D15" s="22" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -921,16 +948,17 @@
       <c r="D17" t="n">
         <v>2.6464</v>
       </c>
-      <c r="E17" t="n">
+      <c r="F17" t="n">
         <v>12.797</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>LOX BAY</t>
         </is>
       </c>
+      <c r="D18" s="22" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -979,16 +1007,17 @@
       <c r="D21" t="n">
         <v>0</v>
       </c>
-      <c r="E21" t="n">
+      <c r="F21" t="n">
         <v>8.387</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
+      <c r="A22" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">AEROCOVER </t>
         </is>
       </c>
+      <c r="D22" s="22" t="n"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1022,7 +1051,8 @@
       <c r="D24" s="6" t="n">
         <v>0.894</v>
       </c>
-      <c r="E24" s="6" t="n">
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n">
         <v>2.379</v>
       </c>
     </row>
@@ -1057,11 +1087,12 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="A27" s="22" t="inlineStr">
         <is>
           <t>PBAY 1</t>
         </is>
       </c>
+      <c r="D27" s="22" t="n"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1110,16 +1141,17 @@
       <c r="D30" t="n">
         <v>1.7528</v>
       </c>
-      <c r="E30" t="n">
+      <c r="F30" t="n">
         <v>17.527</v>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="3" t="inlineStr">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>ETH BAY</t>
         </is>
       </c>
+      <c r="D31" s="22" t="n"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1168,16 +1200,17 @@
       <c r="D34" t="n">
         <v>0</v>
       </c>
-      <c r="E34" t="n">
+      <c r="F34" t="n">
         <v>8.387</v>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="3" t="inlineStr">
+      <c r="A35" s="22" t="inlineStr">
         <is>
           <t>PBAY 2</t>
         </is>
       </c>
+      <c r="D35" s="22" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1226,16 +1259,17 @@
       <c r="D38" t="n">
         <v>1.2154</v>
       </c>
-      <c r="E38" t="n">
+      <c r="F38" t="n">
         <v>14.21</v>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
+      <c r="A39" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">AV BAY </t>
         </is>
       </c>
+      <c r="D39" s="22" t="n"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1269,16 +1303,17 @@
       <c r="D41" t="n">
         <v>0.5427999999999999</v>
       </c>
-      <c r="E41" t="n">
+      <c r="F41" t="n">
         <v>9.835000000000001</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A42" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">RE BAY </t>
         </is>
       </c>
+      <c r="D42" s="22" t="n"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1312,7 +1347,7 @@
       <c r="D44" t="n">
         <v>0.2054</v>
       </c>
-      <c r="E44" t="n">
+      <c r="F44" t="n">
         <v>10.311</v>
       </c>
     </row>
@@ -1362,11 +1397,12 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+      <c r="A48" s="22" t="inlineStr">
         <is>
           <t>NOSE CONE</t>
         </is>
       </c>
+      <c r="D48" s="22" t="n"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1400,16 +1436,17 @@
       <c r="D50" t="n">
         <v>3.683</v>
       </c>
-      <c r="E50" t="n">
+      <c r="F50" t="n">
         <v>5.612</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="3" t="inlineStr">
+      <c r="A51" s="22" t="inlineStr">
         <is>
           <t xml:space="preserve">TANK </t>
         </is>
       </c>
+      <c r="D51" s="22" t="n"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1457,11 +1494,12 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+      <c r="A55" s="22" t="inlineStr">
         <is>
           <t>COPV</t>
         </is>
       </c>
+      <c r="D55" s="22" t="n"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1504,11 +1542,12 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="3" t="inlineStr">
+      <c r="A59" s="22" t="inlineStr">
         <is>
           <t>FINS</t>
         </is>
       </c>
+      <c r="D59" s="22" t="n"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1524,11 +1563,11 @@
           <t>Nombre</t>
         </is>
       </c>
-      <c r="E60">
+      <c r="F60">
         <f>B60*(4.857*B61*((B62+B63)/2))</f>
         <v/>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="G60" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
@@ -1579,7 +1618,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="64" ht="15" customFormat="1" customHeight="1" s="23">
       <c r="A64" t="inlineStr">
         <is>
           <t xml:space="preserve">pos_fins </t>
@@ -1593,11 +1632,11 @@
           <t xml:space="preserve">Position </t>
         </is>
       </c>
-      <c r="E64">
+      <c r="F64">
         <f>(B64-B62)*1000</f>
         <v/>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="G64" t="inlineStr">
         <is>
           <t>mm</t>
         </is>
@@ -1649,11 +1688,12 @@
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="3" t="inlineStr">
+      <c r="A68" s="22" t="inlineStr">
         <is>
           <t>RAIL BUTTON</t>
         </is>
       </c>
+      <c r="D68" s="22" t="n"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1702,15 +1742,15 @@
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A39:C39"/>
     <mergeCell ref="A55:C55"/>
-    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A59:C59"/>
     <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A35:C35"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A51:C51"/>
-    <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="portrait" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
@@ -1721,14 +1761,14 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C40"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.77734375" defaultRowHeight="14.4" customHeight="1" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
-    <col width="32" customWidth="1" style="1" min="1" max="1"/>
-    <col width="16" customWidth="1" style="1" min="2" max="2"/>
-    <col width="55" customWidth="1" style="1" min="3" max="3"/>
+    <col width="32" customWidth="1" style="23" min="1" max="1"/>
+    <col width="16" customWidth="1" style="23" min="2" max="2"/>
+    <col width="55" customWidth="1" style="23" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.05" customFormat="1" customHeight="1" s="1">
+    <row r="1" ht="22.05" customFormat="1" customHeight="1" s="23">
       <c r="A1" s="9" t="inlineStr">
         <is>
           <t>Name</t>
@@ -1746,13 +1786,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="24" t="inlineStr">
         <is>
           <t>PARAMÈTRES</t>
         </is>
       </c>
-      <c r="B2" s="28" t="n"/>
-      <c r="C2" s="28" t="n"/>
+      <c r="B2" s="25" t="n"/>
+      <c r="C2" s="25" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1760,7 +1800,7 @@
           <t>of_ratio</t>
         </is>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="B3" s="10" t="n">
         <v>1.5</v>
       </c>
     </row>
@@ -1770,7 +1810,7 @@
           <t>isp</t>
         </is>
       </c>
-      <c r="B4" s="13" t="n">
+      <c r="B4" s="11" t="n">
         <v>190</v>
       </c>
     </row>
@@ -1780,7 +1820,7 @@
           <t>thrust</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="11" t="n">
         <v>7000</v>
       </c>
       <c r="C5" s="5" t="n"/>
@@ -1791,19 +1831,19 @@
           <t>total_impulse</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="11" t="n">
         <v>36000</v>
       </c>
       <c r="C6" s="5" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="24" t="inlineStr">
         <is>
           <t>MASS FLOW RATE</t>
         </is>
       </c>
-      <c r="B7" s="28" t="n"/>
-      <c r="C7" s="28" t="n"/>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="25" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1811,7 +1851,7 @@
           <t>lox_boil_off</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n">
+      <c r="B8" s="12" t="n">
         <v>0.001</v>
       </c>
     </row>
@@ -1821,7 +1861,7 @@
           <t xml:space="preserve">lox_prechill </t>
         </is>
       </c>
-      <c r="B9" s="15" t="n">
+      <c r="B9" s="13" t="n">
         <v>3.634769409</v>
       </c>
     </row>
@@ -1831,7 +1871,7 @@
           <t>lox_ignition</t>
         </is>
       </c>
-      <c r="B10" s="15" t="n">
+      <c r="B10" s="13" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1841,7 +1881,7 @@
           <t>lox_ramp_up</t>
         </is>
       </c>
-      <c r="B11" s="15" t="n">
+      <c r="B11" s="13" t="n">
         <v>2.623168871</v>
       </c>
     </row>
@@ -1851,7 +1891,7 @@
           <t>lox_ramp_down</t>
         </is>
       </c>
-      <c r="B12" s="15" t="n">
+      <c r="B12" s="13" t="n">
         <v>2.623168871</v>
       </c>
     </row>
@@ -1861,10 +1901,10 @@
           <t>lox_cutoff</t>
         </is>
       </c>
-      <c r="B13" s="15" t="n">
+      <c r="B13" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="15" t="n">
+      <c r="C13" s="13" t="n">
         <v>3.634769409</v>
       </c>
     </row>
@@ -1874,7 +1914,7 @@
           <t xml:space="preserve">eth_ignition </t>
         </is>
       </c>
-      <c r="B14" s="15" t="n">
+      <c r="B14" s="13" t="n">
         <v>2.29321782</v>
       </c>
     </row>
@@ -1884,7 +1924,7 @@
           <t>eth_ramp_up</t>
         </is>
       </c>
-      <c r="B15" s="15" t="n">
+      <c r="B15" s="13" t="n">
         <v>1.672500989</v>
       </c>
     </row>
@@ -1894,7 +1934,7 @@
           <t>eth_ramp_down</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="13" t="n">
         <v>1.672500989</v>
       </c>
     </row>
@@ -1919,13 +1959,13 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>MASS</t>
         </is>
       </c>
-      <c r="B19" s="28" t="n"/>
-      <c r="C19" s="28" t="n"/>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="25" t="n"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1963,7 +2003,7 @@
           <t>eth_pressure</t>
         </is>
       </c>
-      <c r="B22" s="16" t="n">
+      <c r="B22" s="14" t="n">
         <v>6000000</v>
       </c>
       <c r="C22" s="5" t="inlineStr">
@@ -2023,7 +2063,7 @@
           <t>lox_pressure</t>
         </is>
       </c>
-      <c r="B26" s="16" t="n">
+      <c r="B26" s="14" t="n">
         <v>6000000</v>
       </c>
       <c r="C26" s="5" t="inlineStr">
@@ -2032,7 +2072,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="27" ht="15" customFormat="1" customHeight="1" s="23">
       <c r="A27" t="inlineStr">
         <is>
           <t>m_n2</t>
@@ -2048,13 +2088,13 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="10" t="inlineStr">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>TIME</t>
         </is>
       </c>
-      <c r="B28" s="28" t="n"/>
-      <c r="C28" s="28" t="n"/>
+      <c r="B28" s="25" t="n"/>
+      <c r="C28" s="25" t="n"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2117,13 +2157,13 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="10" t="inlineStr">
+      <c r="A35" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">FORCE </t>
         </is>
       </c>
-      <c r="B35" s="28" t="n"/>
-      <c r="C35" s="28" t="n"/>
+      <c r="B35" s="25" t="n"/>
+      <c r="C35" s="25" t="n"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -2156,7 +2196,7 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="17" t="inlineStr">
+      <c r="A38" s="26" t="inlineStr">
         <is>
           <t>THRUST CURVE MODEL</t>
         </is>
@@ -2199,7 +2239,7 @@
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" horizontalDpi="0" verticalDpi="0" copies="1"/>
+  <pageSetup orientation="portrait" paperSize="9" useFirstPageNumber="1" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -2210,38 +2250,38 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C32"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="8.77734375" defaultRowHeight="14.4" customHeight="1" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
-    <col width="32" customWidth="1" style="1" min="1" max="1"/>
-    <col width="16" customWidth="1" style="1" min="2" max="2"/>
-    <col width="55" customWidth="1" style="1" min="3" max="3"/>
+    <col width="32" customWidth="1" style="23" min="1" max="1"/>
+    <col width="16" customWidth="1" style="23" min="2" max="2"/>
+    <col width="55" customWidth="1" style="23" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.05" customFormat="1" customHeight="1" s="1">
-      <c r="A1" s="18" t="inlineStr">
+    <row r="1" ht="22.05" customFormat="1" customHeight="1" s="23">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="19" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">ENREGISTREMENT </t>
         </is>
       </c>
-      <c r="B2" s="28" t="n"/>
-      <c r="C2" s="28" t="n"/>
+      <c r="B2" s="25" t="n"/>
+      <c r="C2" s="25" t="n"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2283,7 +2323,7 @@
           <t>n_points</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
+      <c r="B5" s="11" t="n">
         <v>1000</v>
       </c>
       <c r="C5" s="5" t="inlineStr">
@@ -2310,13 +2350,13 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="27" t="inlineStr">
         <is>
           <t xml:space="preserve">ENVIRONNEMENT </t>
         </is>
       </c>
-      <c r="B7" s="28" t="n"/>
-      <c r="C7" s="28" t="n"/>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="25" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2414,13 +2454,13 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="19" t="inlineStr">
+      <c r="A16" s="27" t="inlineStr">
         <is>
           <t>RAIL</t>
         </is>
       </c>
-      <c r="B16" s="28" t="n"/>
-      <c r="C16" s="28" t="n"/>
+      <c r="B16" s="25" t="n"/>
+      <c r="C16" s="25" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2452,7 +2492,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customFormat="1" customHeight="1" s="1">
+    <row r="19" ht="15" customFormat="1" customHeight="1" s="23">
       <c r="A19" t="inlineStr">
         <is>
           <t>l_rail</t>
@@ -2610,55 +2650,55 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:AC41"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="10.6640625" defaultRowHeight="14.4" customHeight="1" outlineLevelRow="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
-    <col width="22.109375" customWidth="1" style="1" min="1" max="1"/>
-    <col width="35.77734375" customWidth="1" style="1" min="2" max="2"/>
-    <col width="15" customWidth="1" style="1" min="8" max="8"/>
-    <col width="14.88671875" customWidth="1" style="1" min="9" max="9"/>
-    <col width="12.33203125" customWidth="1" style="1" min="29" max="29"/>
+    <col width="22.109375" customWidth="1" style="23" min="1" max="1"/>
+    <col width="35.77734375" customWidth="1" style="23" min="2" max="2"/>
+    <col width="15" customWidth="1" style="23" min="8" max="8"/>
+    <col width="14.88671875" customWidth="1" style="23" min="9" max="9"/>
+    <col width="12.33203125" customWidth="1" style="23" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="12" t="n"/>
-      <c r="B1" s="12" t="n"/>
+      <c r="A1" s="10" t="n"/>
+      <c r="B1" s="10" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="20" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>MASSE</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Dry mass [kg]</t>
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>99.19800000000001</v>
+        <v>98.88979999999999</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Wet mass (initial) [kg]</t>
         </is>
       </c>
       <c r="B4" s="6" t="n">
-        <v>127.4186367881205</v>
+        <v>127.1104367881205</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>PERFORMANCES MOTEUR</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Max thrust [N]</t>
         </is>
@@ -2668,7 +2708,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Total impulse [Ns]</t>
         </is>
@@ -2678,206 +2718,206 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>CINÉMATIQUE &amp; TRAJECTOIRE</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Apogee AGL [m]</t>
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>3145.292549799305</v>
+        <v>3145.375757533603</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Apogee ASL [m]</t>
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>3312.292549799306</v>
+        <v>3296.375757533603</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Max velocity [m/s]</t>
         </is>
       </c>
       <c r="B11" s="6" t="n">
-        <v>250.2159009477571</v>
+        <v>250.9526073078034</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Max acceleration [m/s^2]</t>
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>120.1433105797428</v>
+        <v>139.1683649298294</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Max Mach [-]</t>
         </is>
       </c>
-      <c r="B13" s="22" t="n">
-        <v>0.7355380303891562</v>
+      <c r="B13" s="17" t="n">
+        <v>0.7266701458833361</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Time to apogee [s]</t>
         </is>
       </c>
       <c r="B14" s="6" t="n">
-        <v>27.0745685089398</v>
+        <v>27.05924179016276</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Total flight time [s]</t>
         </is>
       </c>
       <c r="B15" s="6" t="n">
-        <v>235.8714869317141</v>
+        <v>234.315371146966</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>SORTIE DE RAMPE</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Rail exit velocity [m/s]</t>
         </is>
       </c>
       <c r="B17" s="6" t="n">
-        <v>32.37735164937891</v>
+        <v>32.43993249692786</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>Static margin rail exit [c]</t>
         </is>
       </c>
-      <c r="B18" s="22" t="n">
-        <v>4.16385784937688</v>
+      <c r="B18" s="17" t="n">
+        <v>4.047493920382416</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="24" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>STABILITÉ</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="inlineStr">
+      <c r="A20" s="18" t="inlineStr">
         <is>
           <t>Static margin liftoff [c]</t>
         </is>
       </c>
-      <c r="B20" s="22" t="n">
-        <v>4.127412293901282</v>
-      </c>
-    </row>
-    <row r="21" ht="14.7" customFormat="1" customHeight="1" s="1">
-      <c r="A21" s="23" t="n"/>
+      <c r="B20" s="17" t="n">
+        <v>4.013504246372449</v>
+      </c>
+    </row>
+    <row r="21" ht="14.7" customFormat="1" customHeight="1" s="23">
+      <c r="A21" s="18" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="n"/>
+      <c r="A22" s="18" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="n"/>
-    </row>
-    <row r="24" ht="14.7" customFormat="1" customHeight="1" s="1">
-      <c r="A24" s="23" t="n"/>
-    </row>
-    <row r="25" ht="14.7" customFormat="1" customHeight="1" s="1">
-      <c r="A25" s="23" t="n"/>
-      <c r="AC25" s="25" t="inlineStr">
+      <c r="A23" s="18" t="n"/>
+    </row>
+    <row r="24" ht="14.7" customFormat="1" customHeight="1" s="23">
+      <c r="A24" s="18" t="n"/>
+    </row>
+    <row r="25" ht="14.7" customFormat="1" customHeight="1" s="23">
+      <c r="A25" s="18" t="n"/>
+      <c r="AC25" s="19" t="inlineStr">
         <is>
           <t>Wet Mass [g]</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="n"/>
-      <c r="AC26" s="26" t="inlineStr">
+      <c r="A26" s="18" t="n"/>
+      <c r="AC26" s="20" t="inlineStr">
         <is>
           <t>7kN</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="n"/>
-      <c r="AC27" s="26" t="inlineStr">
+      <c r="A27" s="18" t="n"/>
+      <c r="AC27" s="20" t="inlineStr">
         <is>
           <t>Estimation</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="16.95" customFormat="1" customHeight="1" s="1">
-      <c r="A28" s="23" t="n"/>
-      <c r="AC28" s="27" t="n">
+    <row r="28" ht="16.95" customFormat="1" customHeight="1" s="23">
+      <c r="A28" s="18" t="n"/>
+      <c r="AC28" s="21" t="n">
         <v>122003</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="23" t="n"/>
-    </row>
-    <row r="30" ht="15.75" customFormat="1" customHeight="1" s="1">
-      <c r="A30" s="23" t="n"/>
+      <c r="A29" s="18" t="n"/>
+    </row>
+    <row r="30" ht="15.75" customFormat="1" customHeight="1" s="23">
+      <c r="A30" s="18" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="23" t="n"/>
+      <c r="A31" s="18" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="23" t="n"/>
+      <c r="A32" s="18" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="23" t="n"/>
+      <c r="A33" s="18" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="23" t="n"/>
-    </row>
-    <row r="35" ht="14.7" customFormat="1" customHeight="1" s="1">
-      <c r="A35" s="23" t="n"/>
+      <c r="A34" s="18" t="n"/>
+    </row>
+    <row r="35" ht="14.7" customFormat="1" customHeight="1" s="23">
+      <c r="A35" s="18" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="23" t="n"/>
+      <c r="A36" s="18" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="23" t="n"/>
+      <c r="A37" s="18" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="23" t="n"/>
+      <c r="A38" s="18" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="23" t="n"/>
+      <c r="A39" s="18" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="23" t="n"/>
+      <c r="A40" s="18" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="23" t="n"/>
+      <c r="A41" s="18" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>